<commit_message>
fix(excel): fixing dincamic format file as requested
</commit_message>
<xml_diff>
--- a/resources/Formato_Dinamico_.xlsx
+++ b/resources/Formato_Dinamico_.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/santiago/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/santiago/Desktop/creacion activo SAP py/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0831BF54-0CE7-434F-9C7E-DB770D5C8B3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65C90E71-D4EA-874E-B665-80C62C1D563F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="22600" firstSheet="4" activeTab="9" xr2:uid="{CA7242B3-F58B-4D52-905C-F122405A1A29}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="7" xr2:uid="{CA7242B3-F58B-4D52-905C-F122405A1A29}"/>
   </bookViews>
   <sheets>
     <sheet name="Sociedades" sheetId="7" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Criterio " sheetId="2" r:id="rId3"/>
     <sheet name="Ceco" sheetId="3" r:id="rId4"/>
     <sheet name="Emplazamiento" sheetId="4" r:id="rId5"/>
-    <sheet name="_ListasClase" sheetId="8" state="hidden" r:id="rId6"/>
+    <sheet name="_ListasClase" sheetId="8" r:id="rId6"/>
     <sheet name="_Requeridos" sheetId="9" r:id="rId7"/>
     <sheet name="Check list" sheetId="11" r:id="rId8"/>
     <sheet name="Formato" sheetId="5" r:id="rId9"/>
@@ -163,7 +163,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7880" uniqueCount="1532">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7844" uniqueCount="1533">
   <si>
     <t xml:space="preserve">Sociedad </t>
   </si>
@@ -4653,28 +4653,10 @@
     <t>NO</t>
   </si>
   <si>
-    <t>PAÍS</t>
-  </si>
-  <si>
     <t>Preguntas</t>
   </si>
   <si>
     <t>Respuesta</t>
-  </si>
-  <si>
-    <t>¿El activo supera el valor de 1/4 de UIT (Unidad Impositiva Tributaria)?</t>
-  </si>
-  <si>
-    <t>¿Pertenece a un proyecto?</t>
-  </si>
-  <si>
-    <t>¿El equipo va a ser reemplazado en alguna concesión?</t>
-  </si>
-  <si>
-    <t>¿Se compra a través de una orden estadística según tipo de activo (diversos, inmuebles)?</t>
-  </si>
-  <si>
-    <t>¿El activo no está sincronizado AA-PM por la fecha de montaje y esta se reporta al Ministerio/Osinerming?</t>
   </si>
   <si>
     <r>
@@ -4762,9 +4744,6 @@
     <t>Países</t>
   </si>
   <si>
-    <t>¿Es de interés para la organización, de tal forma que esté dispuesta a realizarle seguimiento y control como propiedad, planta y equipo?</t>
-  </si>
-  <si>
     <t>CONFIGURACIÓN PREGUNTAS CHECKLIST POR PAÍS</t>
   </si>
   <si>
@@ -4810,25 +4789,49 @@
     <t>P11</t>
   </si>
   <si>
-    <t>¿El activo es un recurso tangible controlado por la compañía?</t>
-  </si>
-  <si>
-    <t>¿Se espera que el activo sea utilizado en el giro normal del negocio por más de un año?</t>
-  </si>
-  <si>
-    <t>¿Es probable que el activo genere beneficios económicos o apoye funciones administrativas?</t>
-  </si>
-  <si>
-    <t>¿Su valor puede ser medido de forma confiable y razonable?</t>
-  </si>
-  <si>
-    <t>¿El valor del activo supera 2.5 Salarios Mínimos Mensuales Legales Vigentes (SMMLV)?</t>
-  </si>
-  <si>
     <t>¿PUEDE SER CREADO COMO ACTIVO FIJO?</t>
   </si>
   <si>
     <t>UN</t>
+  </si>
+  <si>
+    <t>FILIAL</t>
+  </si>
+  <si>
+    <t>1. ¿El activo es un recurso tangible controlado por la compañía?</t>
+  </si>
+  <si>
+    <t>2. ¿Se espera que el activo sea utilizado en el giro normal del negocio por más de un año?</t>
+  </si>
+  <si>
+    <t>3. ¿Es probable que el activo genere beneficios económicos o apoye funciones administrativas?</t>
+  </si>
+  <si>
+    <t>4. ¿Su valor puede ser medido de forma confiable y razonable?</t>
+  </si>
+  <si>
+    <t>5. ¿El valor del activo supera 2.5 Salarios Mínimos Mensuales Legales Vigentes (SMMLV)?</t>
+  </si>
+  <si>
+    <t>6. ¿Es de interés para la organización, de tal forma que esté dispuesta a realizarle seguimiento y control como propiedad, planta y equipo?</t>
+  </si>
+  <si>
+    <t>7. ¿El activo supera el valor de 1/4 de UIT (Unidad Impositiva Tributaria)?</t>
+  </si>
+  <si>
+    <t>8. ¿El equipo va a ser reemplazado en alguna concesión?</t>
+  </si>
+  <si>
+    <t>9. ¿Pertenece a un proyecto?</t>
+  </si>
+  <si>
+    <t>10. ¿Se compra a través de una orden estadística según tipo de activo (diversos, inmuebles)?</t>
+  </si>
+  <si>
+    <t>11. ¿El activo no está sincronizado AA-PM por la fecha de montaje y esta se reporta al Ministerio/Osinerming?</t>
+  </si>
+  <si>
+    <t>EXCLUSIVO PARA FILIALES DE PERÚ</t>
   </si>
 </sst>
 </file>
@@ -5638,6 +5641,21 @@
     </xf>
     <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -5670,28 +5688,39 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 4" xfId="1" xr:uid="{3283983A-646C-44C7-A2FC-29FE31B28852}"/>
     <cellStyle name="Porcentaje 2" xfId="2" xr:uid="{57290B1F-A1BC-40FC-80FE-1CB63CCFCBB6}"/>
   </cellStyles>
-  <dxfs count="16">
+  <dxfs count="18">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF006400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -5889,13 +5918,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>31750</xdr:colOff>
-      <xdr:row>42</xdr:row>
+      <xdr:row>37</xdr:row>
       <xdr:rowOff>69850</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>655875</xdr:colOff>
-      <xdr:row>53</xdr:row>
+      <xdr:row>48</xdr:row>
       <xdr:rowOff>91838</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -6671,7 +6700,7 @@
         <v>0</v>
       </c>
       <c r="J2" t="s">
-        <v>1531</v>
+        <v>1519</v>
       </c>
       <c r="Q2">
         <f>Formato!N22</f>
@@ -16894,7 +16923,7 @@
         <v>941</v>
       </c>
       <c r="J192" t="s">
-        <v>1506</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="193" spans="1:4" x14ac:dyDescent="0.2">
@@ -42087,7 +42116,7 @@
         <v>1380</v>
       </c>
       <c r="Q1" s="11" t="s">
-        <v>1508</v>
+        <v>1502</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.2">
@@ -45046,7 +45075,7 @@
   <sheetPr codeName="Sheet7">
     <tabColor theme="4" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:Z38"/>
+  <dimension ref="A1:Z23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="102.1640625" bestFit="1" customWidth="1"/>
@@ -45417,55 +45446,55 @@
     </row>
     <row r="16" spans="1:26" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="77" t="s">
-        <v>1510</v>
+        <v>1503</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" s="78" t="s">
-        <v>1511</v>
+        <v>1504</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" s="78" t="s">
-        <v>1512</v>
+        <v>1505</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" s="18" t="s">
+        <v>1506</v>
+      </c>
+      <c r="B20" s="18" t="s">
+        <v>1507</v>
+      </c>
+      <c r="C20" s="18" t="s">
+        <v>1508</v>
+      </c>
+      <c r="D20" s="18" t="s">
+        <v>1509</v>
+      </c>
+      <c r="E20" s="18" t="s">
+        <v>1510</v>
+      </c>
+      <c r="F20" s="18" t="s">
+        <v>1511</v>
+      </c>
+      <c r="G20" s="18" t="s">
+        <v>1512</v>
+      </c>
+      <c r="H20" s="18" t="s">
         <v>1513</v>
       </c>
-      <c r="B20" s="18" t="s">
+      <c r="I20" s="18" t="s">
         <v>1514</v>
       </c>
-      <c r="C20" s="18" t="s">
+      <c r="J20" s="18" t="s">
         <v>1515</v>
       </c>
-      <c r="D20" s="18" t="s">
+      <c r="K20" s="18" t="s">
         <v>1516</v>
       </c>
-      <c r="E20" s="18" t="s">
+      <c r="L20" s="18" t="s">
         <v>1517</v>
-      </c>
-      <c r="F20" s="18" t="s">
-        <v>1518</v>
-      </c>
-      <c r="G20" s="18" t="s">
-        <v>1519</v>
-      </c>
-      <c r="H20" s="18" t="s">
-        <v>1520</v>
-      </c>
-      <c r="I20" s="18" t="s">
-        <v>1521</v>
-      </c>
-      <c r="J20" s="18" t="s">
-        <v>1522</v>
-      </c>
-      <c r="K20" s="18" t="s">
-        <v>1523</v>
-      </c>
-      <c r="L20" s="18" t="s">
-        <v>1524</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.2">
@@ -45547,174 +45576,6 @@
       <c r="J23" s="4"/>
       <c r="K23" s="4"/>
       <c r="L23" s="4"/>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
-        <v>1497</v>
-      </c>
-      <c r="B27" t="s">
-        <v>1441</v>
-      </c>
-      <c r="C27" t="s">
-        <v>1446</v>
-      </c>
-      <c r="D27" t="s">
-        <v>1442</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
-        <v>1525</v>
-      </c>
-      <c r="B28" t="s">
-        <v>1489</v>
-      </c>
-      <c r="C28" t="s">
-        <v>1495</v>
-      </c>
-      <c r="D28" t="s">
-        <v>1489</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
-        <v>1526</v>
-      </c>
-      <c r="B29" t="s">
-        <v>1489</v>
-      </c>
-      <c r="C29" t="s">
-        <v>1495</v>
-      </c>
-      <c r="D29" t="s">
-        <v>1489</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
-        <v>1527</v>
-      </c>
-      <c r="B30" t="s">
-        <v>1489</v>
-      </c>
-      <c r="C30" t="s">
-        <v>1495</v>
-      </c>
-      <c r="D30" t="s">
-        <v>1489</v>
-      </c>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
-        <v>1528</v>
-      </c>
-      <c r="B31" t="s">
-        <v>1489</v>
-      </c>
-      <c r="C31" t="s">
-        <v>1495</v>
-      </c>
-      <c r="D31" t="s">
-        <v>1489</v>
-      </c>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
-        <v>1529</v>
-      </c>
-      <c r="B32" t="s">
-        <v>1489</v>
-      </c>
-      <c r="C32" t="s">
-        <v>1495</v>
-      </c>
-      <c r="D32" t="s">
-        <v>1495</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A33" t="s">
-        <v>1509</v>
-      </c>
-      <c r="B33" t="s">
-        <v>1489</v>
-      </c>
-      <c r="C33" t="s">
-        <v>1495</v>
-      </c>
-      <c r="D33" t="s">
-        <v>1489</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
-        <v>1499</v>
-      </c>
-      <c r="B34" t="s">
-        <v>1495</v>
-      </c>
-      <c r="C34" t="s">
-        <v>1489</v>
-      </c>
-      <c r="D34" t="s">
-        <v>1495</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
-        <v>1501</v>
-      </c>
-      <c r="B35" t="s">
-        <v>1495</v>
-      </c>
-      <c r="C35" t="s">
-        <v>1489</v>
-      </c>
-      <c r="D35" t="s">
-        <v>1495</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
-        <v>1500</v>
-      </c>
-      <c r="B36" t="s">
-        <v>1495</v>
-      </c>
-      <c r="C36" t="s">
-        <v>1489</v>
-      </c>
-      <c r="D36" t="s">
-        <v>1495</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A37" t="s">
-        <v>1502</v>
-      </c>
-      <c r="B37" t="s">
-        <v>1495</v>
-      </c>
-      <c r="C37" t="s">
-        <v>1489</v>
-      </c>
-      <c r="D37" t="s">
-        <v>1495</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A38" t="s">
-        <v>1503</v>
-      </c>
-      <c r="B38" t="s">
-        <v>1495</v>
-      </c>
-      <c r="C38" t="s">
-        <v>1489</v>
-      </c>
-      <c r="D38" t="s">
-        <v>1495</v>
-      </c>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -45734,7 +45595,7 @@
   <sheetPr codeName="Sheet8">
     <tabColor theme="3" tint="0.249977111117893"/>
   </sheetPr>
-  <dimension ref="B4:L42"/>
+  <dimension ref="B4:L37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="1.1640625" customWidth="1"/>
@@ -45745,10 +45606,10 @@
   <sheetData>
     <row r="4" spans="2:12" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="5" spans="2:12" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="F5" s="88" t="s">
+      <c r="F5" s="80" t="s">
         <v>1490</v>
       </c>
-      <c r="G5" s="89"/>
+      <c r="G5" s="81"/>
     </row>
     <row r="6" spans="2:12" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="F6" s="53"/>
@@ -45759,10 +45620,10 @@
       <c r="G7" s="54"/>
     </row>
     <row r="8" spans="2:12" ht="23" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="90" t="s">
+      <c r="B8" s="82" t="s">
         <v>1491</v>
       </c>
-      <c r="C8" s="91"/>
+      <c r="C8" s="83"/>
       <c r="F8" s="25" t="s">
         <v>1492</v>
       </c>
@@ -45787,18 +45648,18 @@
       </c>
     </row>
     <row r="11" spans="2:12" ht="20" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="92" t="s">
-        <v>1505</v>
-      </c>
-      <c r="C11" s="92"/>
+      <c r="B11" s="84" t="s">
+        <v>1499</v>
+      </c>
+      <c r="C11" s="84"/>
       <c r="F11" s="29"/>
       <c r="G11" s="30"/>
     </row>
     <row r="12" spans="2:12" ht="19" x14ac:dyDescent="0.2">
-      <c r="B12" s="92" t="s">
-        <v>1504</v>
-      </c>
-      <c r="C12" s="92"/>
+      <c r="B12" s="84" t="s">
+        <v>1498</v>
+      </c>
+      <c r="C12" s="84"/>
       <c r="L12" s="31" t="s">
         <v>1489</v>
       </c>
@@ -45810,10 +45671,10 @@
     </row>
     <row r="14" spans="2:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B14" s="49" t="s">
-        <v>1496</v>
+        <v>1520</v>
       </c>
       <c r="C14" s="50" t="s">
-        <v>1441</v>
+        <v>64</v>
       </c>
     </row>
     <row r="16" spans="2:12" ht="16" thickBot="1" x14ac:dyDescent="0.25">
@@ -45821,17 +45682,16 @@
     </row>
     <row r="17" spans="2:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B17" s="51" t="s">
+        <v>1496</v>
+      </c>
+      <c r="C17" s="51" t="s">
         <v>1497</v>
       </c>
-      <c r="C17" s="51" t="s">
-        <v>1498</v>
-      </c>
       <c r="L17" s="33"/>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B18" t="str">
-        <f>IF(IFERROR(_xlfn.XLOOKUP('Check list'!$C$14,_Requeridos!$B$27:$D$27,_Requeridos!$B28:$D28,""),"")="SI",_Requeridos!$A28,"")</f>
-        <v>¿El activo es un recurso tangible controlado por la compañía?</v>
+      <c r="B18" t="s">
+        <v>1521</v>
       </c>
       <c r="C18" t="s">
         <v>1489</v>
@@ -45839,9 +45699,8 @@
       <c r="L18" s="33"/>
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B19" t="str">
-        <f>IF(IFERROR(_xlfn.XLOOKUP('Check list'!$C$14,_Requeridos!$B$27:$D$27,_Requeridos!$B29:$D29,""),"")="SI",_Requeridos!$A29,"")</f>
-        <v>¿Se espera que el activo sea utilizado en el giro normal del negocio por más de un año?</v>
+      <c r="B19" t="s">
+        <v>1522</v>
       </c>
       <c r="C19" t="s">
         <v>1489</v>
@@ -45849,9 +45708,8 @@
       <c r="L19" s="33"/>
     </row>
     <row r="20" spans="2:12" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B20" t="str">
-        <f>IF(IFERROR(_xlfn.XLOOKUP('Check list'!$C$14,_Requeridos!$B$27:$D$27,_Requeridos!$B30:$D30,""),"")="SI",_Requeridos!$A30,"")</f>
-        <v>¿Es probable que el activo genere beneficios económicos o apoye funciones administrativas?</v>
+      <c r="B20" t="s">
+        <v>1523</v>
       </c>
       <c r="C20" t="s">
         <v>1489</v>
@@ -45859,116 +45717,124 @@
       <c r="L20" s="32"/>
     </row>
     <row r="21" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B21" t="str">
-        <f>IF(IFERROR(_xlfn.XLOOKUP('Check list'!$C$14,_Requeridos!$B$27:$D$27,_Requeridos!$B31:$D31,""),"")="SI",_Requeridos!$A31,"")</f>
-        <v>¿Su valor puede ser medido de forma confiable y razonable?</v>
+      <c r="B21" t="s">
+        <v>1524</v>
       </c>
       <c r="C21" t="s">
         <v>1489</v>
       </c>
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B22" t="str">
-        <f>IF(IFERROR(_xlfn.XLOOKUP('Check list'!$C$14,_Requeridos!$B$27:$D$27,_Requeridos!$B32:$D32,""),"")="SI",_Requeridos!$A32,"")</f>
-        <v>¿El valor del activo supera 2.5 Salarios Mínimos Mensuales Legales Vigentes (SMMLV)?</v>
+      <c r="B22" t="s">
+        <v>1525</v>
       </c>
       <c r="C22" t="s">
         <v>1489</v>
       </c>
     </row>
     <row r="23" spans="2:12" ht="32" x14ac:dyDescent="0.2">
-      <c r="B23" s="34" t="str">
-        <f>IF(IFERROR(_xlfn.XLOOKUP('Check list'!$C$14,_Requeridos!$B$27:$D$27,_Requeridos!$B33:$D33,""),"")="SI",_Requeridos!$A33,"")</f>
-        <v>¿Es de interés para la organización, de tal forma que esté dispuesta a realizarle seguimiento y control como propiedad, planta y equipo?</v>
+      <c r="B23" s="34" t="s">
+        <v>1526</v>
       </c>
       <c r="C23" t="s">
         <v>1489</v>
       </c>
     </row>
-    <row r="24" spans="2:12" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="47" t="str">
-        <f>IF(IFERROR(_xlfn.XLOOKUP('Check list'!$C$14,_Requeridos!$B$27:$D$27,_Requeridos!$B34:$D34,""),"")="SI",_Requeridos!$A34,"")</f>
-        <v/>
-      </c>
-      <c r="C24" s="47" t="s">
-        <v>1489</v>
-      </c>
-    </row>
-    <row r="25" spans="2:12" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="47" t="str">
-        <f>IF(IFERROR(_xlfn.XLOOKUP('Check list'!$C$14,_Requeridos!$B$27:$D$27,_Requeridos!$B35:$D35,""),"")="SI",_Requeridos!$A35,"")</f>
-        <v/>
-      </c>
-      <c r="C25" s="47" t="s">
-        <v>1489</v>
-      </c>
-    </row>
-    <row r="26" spans="2:12" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="47" t="str">
-        <f>IF(IFERROR(_xlfn.XLOOKUP('Check list'!$C$14,_Requeridos!$B$27:$D$27,_Requeridos!$B36:$D36,""),"")="SI",_Requeridos!$A36,"")</f>
-        <v/>
-      </c>
-      <c r="C26" s="47" t="s">
-        <v>1489</v>
-      </c>
-    </row>
-    <row r="27" spans="2:12" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B27" s="47" t="str">
-        <f>IF(IFERROR(_xlfn.XLOOKUP('Check list'!$C$14,_Requeridos!$B$27:$D$27,_Requeridos!$B37:$D37,""),"")="SI",_Requeridos!$A37,"")</f>
-        <v/>
-      </c>
-      <c r="C27" s="47" t="s">
-        <v>1489</v>
-      </c>
-    </row>
-    <row r="28" spans="2:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B28" s="48" t="str">
-        <f>IF(IFERROR(_xlfn.XLOOKUP('Check list'!$C$14,_Requeridos!$B$27:$D$27,_Requeridos!$B38:$D38,""),"")="SI",_Requeridos!$A38,"")</f>
-        <v/>
+    <row r="25" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B25" s="11" t="s">
+        <v>1518</v>
+      </c>
+      <c r="C25" s="21" t="str">
+        <f ca="1">IF(C14="","Seleccione un país válido",IF(COUNTIFS(B18:B32,"&lt;&gt;""",C18:C32,"NO")&gt;0,"NO CUMPLE","CUMPLE"))</f>
+        <v>CUMPLE</v>
+      </c>
+    </row>
+    <row r="26" spans="2:12" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="2:12" ht="23" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B27" s="82" t="s">
+        <v>1532</v>
+      </c>
+      <c r="C27" s="83"/>
+    </row>
+    <row r="28" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B28" s="47" t="s">
+        <v>1527</v>
       </c>
       <c r="C28" s="47" t="s">
         <v>1489</v>
       </c>
     </row>
     <row r="29" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B29" s="34"/>
-    </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B35" s="11" t="s">
+      <c r="B29" s="47" t="s">
+        <v>1528</v>
+      </c>
+      <c r="C29" s="47" t="s">
+        <v>1489</v>
+      </c>
+    </row>
+    <row r="30" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B30" s="47" t="s">
+        <v>1529</v>
+      </c>
+      <c r="C30" s="47" t="s">
+        <v>1489</v>
+      </c>
+    </row>
+    <row r="31" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B31" s="47" t="s">
         <v>1530</v>
       </c>
-      <c r="C35" s="21" t="str">
-        <f>IF(C14="","Seleccione un país válido",IF(COUNTIFS(B18:B28,"&lt;&gt;""",C18:C28,"NO")&gt;0,"NO CUMPLE","CUMPLE"))</f>
+      <c r="C31" s="47" t="s">
+        <v>1489</v>
+      </c>
+    </row>
+    <row r="32" spans="2:12" ht="16" x14ac:dyDescent="0.2">
+      <c r="B32" s="48" t="s">
+        <v>1531</v>
+      </c>
+      <c r="C32" s="47" t="s">
+        <v>1489</v>
+      </c>
+    </row>
+    <row r="34" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="C34" s="21" t="str">
+        <f>IF(C14="","Seleccione un país válido",IF(COUNTIFS(B28:B32,"&lt;&gt;""",C28:C32,"NO")&gt;0,"NO CUMPLE","CUMPLE"))</f>
         <v>CUMPLE</v>
       </c>
     </row>
-    <row r="42" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B42" s="52" t="s">
-        <v>1507</v>
+    <row r="37" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B37" s="52" t="s">
+        <v>1501</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="F5:G5"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B27:C27"/>
   </mergeCells>
-  <conditionalFormatting sqref="C18:C28">
-    <cfRule type="expression" dxfId="4" priority="51">
-      <formula>B18=""</formula>
+  <conditionalFormatting sqref="C25">
+    <cfRule type="containsText" dxfId="5" priority="27" operator="containsText" text="NO CUMPLE">
+      <formula>NOT(ISERROR(SEARCH("NO CUMPLE",C25)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="4" priority="28" operator="containsText" text="CUMPLE">
+      <formula>NOT(ISERROR(SEARCH("CUMPLE",C25)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C35">
-    <cfRule type="containsText" dxfId="3" priority="27" operator="containsText" text="NO CUMPLE">
-      <formula>NOT(ISERROR(SEARCH("NO CUMPLE",C35)))</formula>
+  <conditionalFormatting sqref="C34">
+    <cfRule type="containsText" dxfId="1" priority="29" operator="containsText" text="NO CUMPLE">
+      <formula>NOT(ISERROR(SEARCH("NO CUMPLE",C34)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="28" operator="containsText" text="CUMPLE">
-      <formula>NOT(ISERROR(SEARCH("CUMPLE",C35)))</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C34">
+    <cfRule type="containsText" dxfId="0" priority="30" operator="containsText" text="CUMPLE">
+      <formula>NOT(ISERROR(SEARCH("CUMPLE",C34)))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C13 C15:C16 C18:C29" xr:uid="{59ED7ABD-2EF3-4F7C-8CCB-C3B41B691E96}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C13 C15:C16 C28:C32 C18:C23" xr:uid="{59ED7ABD-2EF3-4F7C-8CCB-C3B41B691E96}">
       <formula1>$L$12:$L$13</formula1>
     </dataValidation>
   </dataValidations>
@@ -45979,202 +45845,11 @@
   </headerFooter>
   <drawing r:id="rId2"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
-      <x14:conditionalFormattings>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="expression" priority="29" id="{C6F7AAB8-2ACB-5948-8914-7B3367303C3F}">
-            <xm:f>IFERROR(_xlfn.XLOOKUP($C$14,_Requeridos!$A$21:$A$30,_Requeridos!$B$21:$B$30,""),"") &lt;&gt; "SI"</xm:f>
-            <x14:dxf>
-              <font>
-                <color rgb="FFFFFFFF"/>
-              </font>
-              <fill>
-                <patternFill patternType="solid">
-                  <fgColor indexed="64"/>
-                  <bgColor rgb="FFFFFFFF"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>B18</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="expression" priority="31" id="{CE08586A-BC88-2A4D-95C4-65DCEFCF42E6}">
-            <xm:f>IFERROR(_xlfn.XLOOKUP($C$14,_Requeridos!$A$21:$A$30,_Requeridos!$C$21:$C$30,""),"") &lt;&gt; "SI"</xm:f>
-            <x14:dxf>
-              <font>
-                <color rgb="FFFFFFFF"/>
-              </font>
-              <fill>
-                <patternFill patternType="solid">
-                  <fgColor indexed="64"/>
-                  <bgColor rgb="FFFFFFFF"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>B19</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="expression" priority="33" id="{A6203441-A068-4A4B-9577-139E76C45968}">
-            <xm:f>IFERROR(_xlfn.XLOOKUP($C$14,_Requeridos!$A$21:$A$30,_Requeridos!$D$21:$D$30,""),"") &lt;&gt; "SI"</xm:f>
-            <x14:dxf>
-              <font>
-                <color rgb="FFFFFFFF"/>
-              </font>
-              <fill>
-                <patternFill patternType="solid">
-                  <fgColor indexed="64"/>
-                  <bgColor rgb="FFFFFFFF"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>B20</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="expression" priority="35" id="{28C7941B-1876-1046-8874-5722020BE513}">
-            <xm:f>IFERROR(_xlfn.XLOOKUP($C$14,_Requeridos!$A$21:$A$30,_Requeridos!$E$21:$E$30,""),"") &lt;&gt; "SI"</xm:f>
-            <x14:dxf>
-              <font>
-                <color rgb="FFFFFFFF"/>
-              </font>
-              <fill>
-                <patternFill patternType="solid">
-                  <fgColor indexed="64"/>
-                  <bgColor rgb="FFFFFFFF"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>B21</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="expression" priority="37" id="{72ACC58B-1D1B-DD46-8B5A-797507531A08}">
-            <xm:f>IFERROR(_xlfn.XLOOKUP($C$14,_Requeridos!$A$21:$A$30,_Requeridos!$F$21:$F$30,""),"") &lt;&gt; "SI"</xm:f>
-            <x14:dxf>
-              <font>
-                <color rgb="FFFFFFFF"/>
-              </font>
-              <fill>
-                <patternFill patternType="solid">
-                  <fgColor indexed="64"/>
-                  <bgColor rgb="FFFFFFFF"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>B22</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="expression" priority="39" id="{CBFFBDF4-04E7-9640-9C89-905137E125AC}">
-            <xm:f>IFERROR(_xlfn.XLOOKUP($C$14,_Requeridos!$A$21:$A$30,_Requeridos!$G$21:$G$30,""),"") &lt;&gt; "SI"</xm:f>
-            <x14:dxf>
-              <font>
-                <color rgb="FFFFFFFF"/>
-              </font>
-              <fill>
-                <patternFill patternType="solid">
-                  <fgColor indexed="64"/>
-                  <bgColor rgb="FFFFFFFF"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>B23</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="expression" priority="41" id="{6F1567CF-EAC7-D742-B3AA-576B12F76461}">
-            <xm:f>IFERROR(_xlfn.XLOOKUP($C$14,_Requeridos!$A$21:$A$30,_Requeridos!$H$21:$H$30,""),"") &lt;&gt; "SI"</xm:f>
-            <x14:dxf>
-              <font>
-                <color rgb="FFFFFFFF"/>
-              </font>
-              <fill>
-                <patternFill patternType="solid">
-                  <fgColor indexed="64"/>
-                  <bgColor rgb="FFFFFFFF"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>B24</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="expression" priority="43" id="{8434A182-8D55-AD4E-9E6D-49DC14BAF881}">
-            <xm:f>IFERROR(_xlfn.XLOOKUP($C$14,_Requeridos!$A$21:$A$30,_Requeridos!$I$21:$I$30,""),"") &lt;&gt; "SI"</xm:f>
-            <x14:dxf>
-              <font>
-                <color rgb="FFFFFFFF"/>
-              </font>
-              <fill>
-                <patternFill patternType="solid">
-                  <fgColor indexed="64"/>
-                  <bgColor rgb="FFFFFFFF"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>B25</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="expression" priority="45" id="{4EF82847-CE1B-4A47-A7C8-A33F1C37F09D}">
-            <xm:f>IFERROR(_xlfn.XLOOKUP($C$14,_Requeridos!$A$21:$A$30,_Requeridos!$J$21:$J$30,""),"") &lt;&gt; "SI"</xm:f>
-            <x14:dxf>
-              <font>
-                <color rgb="FFFFFFFF"/>
-              </font>
-              <fill>
-                <patternFill patternType="solid">
-                  <fgColor indexed="64"/>
-                  <bgColor rgb="FFFFFFFF"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>B26</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="expression" priority="47" id="{EB3BEA08-97F5-3C4D-869B-42212D6D0A52}">
-            <xm:f>IFERROR(_xlfn.XLOOKUP($C$14,_Requeridos!$A$21:$A$30,_Requeridos!$K$21:$K$30,""),"") &lt;&gt; "SI"</xm:f>
-            <x14:dxf>
-              <font>
-                <color rgb="FFFFFFFF"/>
-              </font>
-              <fill>
-                <patternFill patternType="solid">
-                  <fgColor indexed="64"/>
-                  <bgColor rgb="FFFFFFFF"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>B27</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="expression" priority="49" id="{B24B4B04-B24F-8941-8A0D-885423D539B8}">
-            <xm:f>IFERROR(_xlfn.XLOOKUP($C$14,_Requeridos!$A$21:$A$30,_Requeridos!$L$21:$L$30,""),"") &lt;&gt; "SI"</xm:f>
-            <x14:dxf>
-              <font>
-                <color rgb="FFFFFFFF"/>
-              </font>
-              <fill>
-                <patternFill patternType="solid">
-                  <fgColor indexed="64"/>
-                  <bgColor rgb="FFFFFFFF"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>B28</xm:sqref>
-        </x14:conditionalFormatting>
-      </x14:conditionalFormattings>
-    </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="País" prompt="Selecciona el país" xr:uid="{24B190AB-A1BD-9342-A014-8FAC3536C7F8}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B5DB2DB7-FD43-5546-BD62-0D7870E179BD}">
           <x14:formula1>
-            <xm:f>_ListasClase!$Q$2:$Q$10</xm:f>
+            <xm:f>Sociedades!$A$2:$A$10</xm:f>
           </x14:formula1>
           <xm:sqref>C14</xm:sqref>
         </x14:dataValidation>
@@ -46267,81 +45942,81 @@
     </row>
     <row r="11" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A11" s="39"/>
-      <c r="B11" s="82" t="s">
+      <c r="B11" s="87" t="s">
         <v>1348</v>
       </c>
-      <c r="C11" s="83"/>
-      <c r="D11" s="83"/>
-      <c r="E11" s="83"/>
-      <c r="F11" s="83"/>
-      <c r="G11" s="83"/>
-      <c r="H11" s="83"/>
-      <c r="I11" s="83"/>
-      <c r="J11" s="83"/>
-      <c r="K11" s="83"/>
-      <c r="L11" s="83"/>
-      <c r="M11" s="83"/>
-      <c r="N11" s="83"/>
-      <c r="O11" s="83"/>
-      <c r="P11" s="83"/>
-      <c r="Q11" s="83"/>
-      <c r="R11" s="83"/>
-      <c r="S11" s="83"/>
-      <c r="T11" s="83"/>
-      <c r="U11" s="83"/>
-      <c r="V11" s="83"/>
-      <c r="W11" s="83"/>
-      <c r="X11" s="83"/>
-      <c r="Y11" s="83"/>
-      <c r="Z11" s="83"/>
-      <c r="AA11" s="83"/>
-      <c r="AB11" s="83"/>
-      <c r="AC11" s="83"/>
-      <c r="AD11" s="83"/>
-      <c r="AE11" s="83"/>
-      <c r="AF11" s="83"/>
-      <c r="AG11" s="83"/>
-      <c r="AH11" s="83"/>
-      <c r="AI11" s="83"/>
-      <c r="AJ11" s="84"/>
+      <c r="C11" s="88"/>
+      <c r="D11" s="88"/>
+      <c r="E11" s="88"/>
+      <c r="F11" s="88"/>
+      <c r="G11" s="88"/>
+      <c r="H11" s="88"/>
+      <c r="I11" s="88"/>
+      <c r="J11" s="88"/>
+      <c r="K11" s="88"/>
+      <c r="L11" s="88"/>
+      <c r="M11" s="88"/>
+      <c r="N11" s="88"/>
+      <c r="O11" s="88"/>
+      <c r="P11" s="88"/>
+      <c r="Q11" s="88"/>
+      <c r="R11" s="88"/>
+      <c r="S11" s="88"/>
+      <c r="T11" s="88"/>
+      <c r="U11" s="88"/>
+      <c r="V11" s="88"/>
+      <c r="W11" s="88"/>
+      <c r="X11" s="88"/>
+      <c r="Y11" s="88"/>
+      <c r="Z11" s="88"/>
+      <c r="AA11" s="88"/>
+      <c r="AB11" s="88"/>
+      <c r="AC11" s="88"/>
+      <c r="AD11" s="88"/>
+      <c r="AE11" s="88"/>
+      <c r="AF11" s="88"/>
+      <c r="AG11" s="88"/>
+      <c r="AH11" s="88"/>
+      <c r="AI11" s="88"/>
+      <c r="AJ11" s="89"/>
     </row>
     <row r="12" spans="1:36" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="40"/>
-      <c r="B12" s="85"/>
-      <c r="C12" s="86"/>
-      <c r="D12" s="86"/>
-      <c r="E12" s="86"/>
-      <c r="F12" s="86"/>
-      <c r="G12" s="86"/>
-      <c r="H12" s="86"/>
-      <c r="I12" s="86"/>
-      <c r="J12" s="86"/>
-      <c r="K12" s="86"/>
-      <c r="L12" s="86"/>
-      <c r="M12" s="86"/>
-      <c r="N12" s="86"/>
-      <c r="O12" s="86"/>
-      <c r="P12" s="86"/>
-      <c r="Q12" s="86"/>
-      <c r="R12" s="86"/>
-      <c r="S12" s="86"/>
-      <c r="T12" s="86"/>
-      <c r="U12" s="86"/>
-      <c r="V12" s="86"/>
-      <c r="W12" s="86"/>
-      <c r="X12" s="86"/>
-      <c r="Y12" s="86"/>
-      <c r="Z12" s="86"/>
-      <c r="AA12" s="86"/>
-      <c r="AB12" s="86"/>
-      <c r="AC12" s="86"/>
-      <c r="AD12" s="86"/>
-      <c r="AE12" s="86"/>
-      <c r="AF12" s="86"/>
-      <c r="AG12" s="86"/>
-      <c r="AH12" s="86"/>
-      <c r="AI12" s="86"/>
-      <c r="AJ12" s="87"/>
+      <c r="B12" s="90"/>
+      <c r="C12" s="91"/>
+      <c r="D12" s="91"/>
+      <c r="E12" s="91"/>
+      <c r="F12" s="91"/>
+      <c r="G12" s="91"/>
+      <c r="H12" s="91"/>
+      <c r="I12" s="91"/>
+      <c r="J12" s="91"/>
+      <c r="K12" s="91"/>
+      <c r="L12" s="91"/>
+      <c r="M12" s="91"/>
+      <c r="N12" s="91"/>
+      <c r="O12" s="91"/>
+      <c r="P12" s="91"/>
+      <c r="Q12" s="91"/>
+      <c r="R12" s="91"/>
+      <c r="S12" s="91"/>
+      <c r="T12" s="91"/>
+      <c r="U12" s="91"/>
+      <c r="V12" s="91"/>
+      <c r="W12" s="91"/>
+      <c r="X12" s="91"/>
+      <c r="Y12" s="91"/>
+      <c r="Z12" s="91"/>
+      <c r="AA12" s="91"/>
+      <c r="AB12" s="91"/>
+      <c r="AC12" s="91"/>
+      <c r="AD12" s="91"/>
+      <c r="AE12" s="91"/>
+      <c r="AF12" s="91"/>
+      <c r="AG12" s="91"/>
+      <c r="AH12" s="91"/>
+      <c r="AI12" s="91"/>
+      <c r="AJ12" s="92"/>
     </row>
     <row r="13" spans="1:36" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="75"/>
@@ -46389,9 +46064,9 @@
       <c r="C14" s="74" t="s">
         <v>3</v>
       </c>
-      <c r="D14" s="80"/>
-      <c r="E14" s="80"/>
-      <c r="F14" s="80"/>
+      <c r="D14" s="85"/>
+      <c r="E14" s="85"/>
+      <c r="F14" s="85"/>
       <c r="G14" s="56"/>
       <c r="H14" s="60"/>
       <c r="I14" s="60"/>
@@ -46429,9 +46104,9 @@
         <v>1350</v>
       </c>
       <c r="C15" s="56"/>
-      <c r="D15" s="80"/>
-      <c r="E15" s="80"/>
-      <c r="F15" s="80"/>
+      <c r="D15" s="85"/>
+      <c r="E15" s="85"/>
+      <c r="F15" s="85"/>
       <c r="G15" s="56"/>
       <c r="H15" s="60"/>
       <c r="I15" s="60"/>
@@ -46469,9 +46144,9 @@
         <v>1351</v>
       </c>
       <c r="C16" s="57"/>
-      <c r="D16" s="80"/>
-      <c r="E16" s="80"/>
-      <c r="F16" s="80"/>
+      <c r="D16" s="85"/>
+      <c r="E16" s="85"/>
+      <c r="F16" s="85"/>
       <c r="G16" s="61"/>
       <c r="H16" s="60"/>
       <c r="I16" s="60"/>
@@ -46509,9 +46184,9 @@
         <v>1352</v>
       </c>
       <c r="C17" s="59"/>
-      <c r="D17" s="80"/>
-      <c r="E17" s="80"/>
-      <c r="F17" s="80"/>
+      <c r="D17" s="85"/>
+      <c r="E17" s="85"/>
+      <c r="F17" s="85"/>
       <c r="G17" s="61"/>
       <c r="H17" s="60"/>
       <c r="I17" s="60"/>
@@ -46549,9 +46224,9 @@
         <v>1353</v>
       </c>
       <c r="C18" s="59"/>
-      <c r="D18" s="80"/>
-      <c r="E18" s="80"/>
-      <c r="F18" s="80"/>
+      <c r="D18" s="85"/>
+      <c r="E18" s="85"/>
+      <c r="F18" s="85"/>
       <c r="G18" s="61"/>
       <c r="H18" s="60"/>
       <c r="I18" s="60"/>
@@ -46589,9 +46264,9 @@
         <v>1354</v>
       </c>
       <c r="C19" s="59"/>
-      <c r="D19" s="80"/>
-      <c r="E19" s="80"/>
-      <c r="F19" s="80"/>
+      <c r="D19" s="85"/>
+      <c r="E19" s="85"/>
+      <c r="F19" s="85"/>
       <c r="G19" s="61"/>
       <c r="H19" s="60"/>
       <c r="I19" s="60"/>
@@ -46656,11 +46331,11 @@
       <c r="AD20" s="37"/>
       <c r="AE20" s="37"/>
       <c r="AF20" s="37"/>
-      <c r="AG20" s="81" t="s">
+      <c r="AG20" s="86" t="s">
         <v>1355</v>
       </c>
-      <c r="AH20" s="81"/>
-      <c r="AI20" s="81"/>
+      <c r="AH20" s="86"/>
+      <c r="AI20" s="86"/>
     </row>
     <row r="21" spans="1:37" s="45" customFormat="1" ht="48.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="43"/>
@@ -50322,10 +49997,10 @@
     <mergeCell ref="B11:AJ12"/>
   </mergeCells>
   <conditionalFormatting sqref="AJ22:AJ89">
-    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Faltan">
+    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Faltan">
       <formula>NOT(ISERROR(SEARCH("Faltan",AJ22)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="Completo">
+    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="Completo">
       <formula>NOT(ISERROR(SEARCH("Completo",AJ22)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>